<commit_message>
Corrige marcação da Ponte Sumaúma: eixo km 661 vs vão OSM
O ponto BQ railway_km_661 fica no aterro (~170 m a oeste do vão).
Mapa passa a exibir Km 661 (eixo) e Ponte Sumaúma (vão ~km 660,8).

Co-authored-by: gabrielavitelli <gabrielavitelli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EFC_nivel_pontos_resumo.xlsx
+++ b/EFC_nivel_pontos_resumo.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,12 +568,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sumauma</t>
+          <t>km661_eixo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ponte Sumaúma (Km 661)</t>
+          <t>Km 661 (eixo)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EFC (railway_km_661)</t>
+          <t>BQ railway_km_661 (quilometragem no eixo)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -596,6 +596,42 @@
         <v>661</v>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>EWS6971 - Abrigo km 663.xlsx (EWS mais próximo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sumauma_vao</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ponte Sumaúma (vão)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>-5.149460125</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-48.375528475</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OSM bridge EFC ways 309747856+1069345405 (mid dual-track)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EWS6971</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>660.83</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>EWS6971 - Abrigo km 663.xlsx (EWS mais próximo)</t>
         </is>
@@ -612,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -816,12 +852,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ponte Sumaúma (Km 661)</t>
+          <t>Km 661 (eixo)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EFC (railway_km_661)</t>
+          <t>BQ railway_km_661 (quilometragem no eixo)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -857,6 +893,53 @@
         </is>
       </c>
       <c r="K5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ponte Sumaúma (vão)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>OSM bridge EFC ways 309747856+1069345405 (mid dual-track)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EWS6971</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>-5.149460125</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-48.375528475</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ANA · RIO TOCANTINS - SÃO SEBASTIÃO DO TO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>23800495</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2639,7 +2722,7 @@
         <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>